<commit_message>
Ajout règle de gestion sur l'idPDV efd0dc60ff6140594727efb62a05985a0d69b8b0
</commit_message>
<xml_diff>
--- a/448-contenu-fhir---ajout-du-projet-de-vie/ig/StructureDefinition-tddui-goal-projet-vie.xlsx
+++ b/448-contenu-fhir---ajout-du-projet-de-vie/ig/StructureDefinition-tddui-goal-projet-vie.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2385" uniqueCount="464">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2385" uniqueCount="465">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-11T14:21:35+00:00</t>
+    <t>2026-06-11T15:13:29+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -669,6 +669,10 @@
   </si>
   <si>
     <t>External Ids for this goal</t>
+  </si>
+  <si>
+    <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
+GoalProjetVieIdentifierFormat:l'identifiant du projet de vie doit respecter le format :  3+FINESS/identifiantLocalUsagerESSMS-PDV-idLocalProjetVie {value.matches('^3[0-9]{9}/[A-Za-z0-9]+-PDV-[A-Za-z0-9]+$')}</t>
   </si>
   <si>
     <t>Goal.identifier:idPDV.id</t>
@@ -4076,7 +4080,7 @@
         <v>77</v>
       </c>
       <c r="AJ20" t="s" s="2">
-        <v>101</v>
+        <v>211</v>
       </c>
       <c r="AK20" t="s" s="2">
         <v>77</v>
@@ -4093,10 +4097,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -4205,10 +4209,10 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -4319,10 +4323,10 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -4348,16 +4352,16 @@
         <v>166</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="N23" t="s" s="2">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="O23" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="P23" t="s" s="2">
         <v>77</v>
@@ -4382,13 +4386,13 @@
         <v>77</v>
       </c>
       <c r="X23" t="s" s="2">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="Y23" t="s" s="2">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="Z23" t="s" s="2">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>77</v>
@@ -4406,7 +4410,7 @@
         <v>77</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>78</v>
@@ -4427,7 +4431,7 @@
         <v>189</v>
       </c>
       <c r="AM23" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="AN23" t="s" s="2">
         <v>77</v>
@@ -4435,10 +4439,10 @@
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4461,19 +4465,19 @@
         <v>90</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="N24" t="s" s="2">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="O24" t="s" s="2">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="P24" t="s" s="2">
         <v>77</v>
@@ -4483,7 +4487,7 @@
         <v>77</v>
       </c>
       <c r="S24" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="T24" t="s" s="2">
         <v>77</v>
@@ -4501,10 +4505,10 @@
         <v>148</v>
       </c>
       <c r="Y24" t="s" s="2">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="Z24" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="AA24" t="s" s="2">
         <v>77</v>
@@ -4522,7 +4526,7 @@
         <v>77</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>78</v>
@@ -4540,10 +4544,10 @@
         <v>77</v>
       </c>
       <c r="AL24" t="s" s="2">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="AM24" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="AN24" t="s" s="2">
         <v>77</v>
@@ -4551,10 +4555,10 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4580,16 +4584,16 @@
         <v>132</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="N25" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="O25" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="P25" t="s" s="2">
         <v>77</v>
@@ -4599,10 +4603,10 @@
         <v>77</v>
       </c>
       <c r="S25" t="s" s="2">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="T25" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="U25" t="s" s="2">
         <v>77</v>
@@ -4638,7 +4642,7 @@
         <v>77</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>78</v>
@@ -4656,10 +4660,10 @@
         <v>77</v>
       </c>
       <c r="AL25" t="s" s="2">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="AM25" t="s" s="2">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="AN25" t="s" s="2">
         <v>77</v>
@@ -4667,10 +4671,10 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4696,13 +4700,13 @@
         <v>103</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="N26" t="s" s="2">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="O26" s="2"/>
       <c r="P26" t="s" s="2">
@@ -4716,7 +4720,7 @@
         <v>77</v>
       </c>
       <c r="T26" t="s" s="2">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="U26" t="s" s="2">
         <v>77</v>
@@ -4752,7 +4756,7 @@
         <v>77</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>78</v>
@@ -4770,10 +4774,10 @@
         <v>77</v>
       </c>
       <c r="AL26" t="s" s="2">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="AM26" t="s" s="2">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="AN26" t="s" s="2">
         <v>77</v>
@@ -4781,10 +4785,10 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4807,13 +4811,13 @@
         <v>90</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -4864,7 +4868,7 @@
         <v>77</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>78</v>
@@ -4882,10 +4886,10 @@
         <v>77</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="AM27" t="s" s="2">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="AN27" t="s" s="2">
         <v>77</v>
@@ -4893,10 +4897,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4919,16 +4923,16 @@
         <v>90</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="N28" t="s" s="2">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
@@ -4978,7 +4982,7 @@
         <v>77</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>78</v>
@@ -4996,10 +5000,10 @@
         <v>77</v>
       </c>
       <c r="AL28" t="s" s="2">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AM28" t="s" s="2">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AN28" t="s" s="2">
         <v>77</v>
@@ -5007,10 +5011,10 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -5036,16 +5040,16 @@
         <v>166</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="N29" t="s" s="2">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="O29" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="P29" t="s" s="2">
         <v>77</v>
@@ -5070,13 +5074,13 @@
         <v>77</v>
       </c>
       <c r="X29" t="s" s="2">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="Y29" t="s" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="Z29" t="s" s="2">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="AA29" t="s" s="2">
         <v>77</v>
@@ -5094,7 +5098,7 @@
         <v>77</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>89</v>
@@ -5109,24 +5113,24 @@
         <v>101</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="AL29" t="s" s="2">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="AM29" t="s" s="2">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="AN29" t="s" s="2">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -5152,10 +5156,10 @@
         <v>103</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
@@ -5235,10 +5239,10 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -5264,10 +5268,10 @@
         <v>110</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -5345,13 +5349,13 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C32" t="s" s="2">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D32" t="s" s="2">
         <v>77</v>
@@ -5373,13 +5377,13 @@
         <v>77</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -5439,13 +5443,13 @@
         <v>79</v>
       </c>
       <c r="AI32" t="s" s="2">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="AJ32" t="s" s="2">
         <v>118</v>
       </c>
       <c r="AK32" t="s" s="2">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="AL32" t="s" s="2">
         <v>77</v>
@@ -5459,10 +5463,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5488,10 +5492,10 @@
         <v>103</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
@@ -5542,7 +5546,7 @@
         <v>77</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>78</v>
@@ -5571,10 +5575,10 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5597,13 +5601,13 @@
         <v>90</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
@@ -5633,10 +5637,10 @@
         <v>170</v>
       </c>
       <c r="Y34" t="s" s="2">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="Z34" t="s" s="2">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="AA34" t="s" s="2">
         <v>77</v>
@@ -5654,7 +5658,7 @@
         <v>77</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>78</v>
@@ -5675,7 +5679,7 @@
         <v>77</v>
       </c>
       <c r="AM34" t="s" s="2">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="AN34" t="s" s="2">
         <v>77</v>
@@ -5683,10 +5687,10 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5709,17 +5713,17 @@
         <v>90</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" t="s" s="2">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="P35" t="s" s="2">
         <v>77</v>
@@ -5747,10 +5751,10 @@
         <v>156</v>
       </c>
       <c r="Y35" t="s" s="2">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="Z35" t="s" s="2">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="AA35" t="s" s="2">
         <v>77</v>
@@ -5768,7 +5772,7 @@
         <v>77</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>78</v>
@@ -5792,15 +5796,15 @@
         <v>77</v>
       </c>
       <c r="AN35" t="s" s="2">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5823,19 +5827,19 @@
         <v>90</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="N36" t="s" s="2">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="O36" t="s" s="2">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="P36" t="s" s="2">
         <v>77</v>
@@ -5863,10 +5867,10 @@
         <v>170</v>
       </c>
       <c r="Y36" t="s" s="2">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="Z36" t="s" s="2">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="AA36" t="s" s="2">
         <v>77</v>
@@ -5884,7 +5888,7 @@
         <v>77</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>78</v>
@@ -5905,18 +5909,18 @@
         <v>77</v>
       </c>
       <c r="AM36" t="s" s="2">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="AN36" t="s" s="2">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -5939,19 +5943,19 @@
         <v>90</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="N37" t="s" s="2">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="O37" t="s" s="2">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="P37" t="s" s="2">
         <v>77</v>
@@ -5979,10 +5983,10 @@
         <v>156</v>
       </c>
       <c r="Y37" t="s" s="2">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="Z37" t="s" s="2">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="AA37" t="s" s="2">
         <v>77</v>
@@ -6000,7 +6004,7 @@
         <v>77</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>89</v>
@@ -6018,21 +6022,21 @@
         <v>77</v>
       </c>
       <c r="AL37" t="s" s="2">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="AM37" t="s" s="2">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="AN37" t="s" s="2">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -6141,10 +6145,10 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -6255,10 +6259,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6284,16 +6288,16 @@
         <v>144</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="N40" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="O40" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="P40" t="s" s="2">
         <v>77</v>
@@ -6342,7 +6346,7 @@
         <v>77</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>78</v>
@@ -6360,10 +6364,10 @@
         <v>77</v>
       </c>
       <c r="AL40" t="s" s="2">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="AM40" t="s" s="2">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="AN40" t="s" s="2">
         <v>77</v>
@@ -6371,10 +6375,10 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6400,16 +6404,16 @@
         <v>103</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="N41" t="s" s="2">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="O41" t="s" s="2">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="P41" t="s" s="2">
         <v>77</v>
@@ -6458,7 +6462,7 @@
         <v>77</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>78</v>
@@ -6473,13 +6477,13 @@
         <v>101</v>
       </c>
       <c r="AK41" t="s" s="2">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="AL41" t="s" s="2">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="AM41" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="AN41" t="s" s="2">
         <v>77</v>
@@ -6487,10 +6491,10 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6513,17 +6517,17 @@
         <v>90</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" t="s" s="2">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="P42" t="s" s="2">
         <v>77</v>
@@ -6572,7 +6576,7 @@
         <v>77</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>89</v>
@@ -6587,24 +6591,24 @@
         <v>101</v>
       </c>
       <c r="AK42" t="s" s="2">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="AL42" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="AM42" t="s" s="2">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="AN42" t="s" s="2">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6627,17 +6631,17 @@
         <v>90</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="N43" s="2"/>
       <c r="O43" t="s" s="2">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P43" t="s" s="2">
         <v>77</v>
@@ -6665,16 +6669,16 @@
         <v>156</v>
       </c>
       <c r="Y43" t="s" s="2">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="Z43" t="s" s="2">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="AA43" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AB43" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="AC43" s="2"/>
       <c r="AD43" t="s" s="2">
@@ -6684,7 +6688,7 @@
         <v>116</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>78</v>
@@ -6708,18 +6712,18 @@
         <v>77</v>
       </c>
       <c r="AN43" t="s" s="2">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C44" t="s" s="2">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="D44" t="s" s="2">
         <v>77</v>
@@ -6741,17 +6745,17 @@
         <v>90</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="N44" s="2"/>
       <c r="O44" t="s" s="2">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P44" t="s" s="2">
         <v>77</v>
@@ -6800,7 +6804,7 @@
         <v>77</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>78</v>
@@ -6815,7 +6819,7 @@
         <v>101</v>
       </c>
       <c r="AK44" t="s" s="2">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="AL44" t="s" s="2">
         <v>77</v>
@@ -6824,15 +6828,15 @@
         <v>77</v>
       </c>
       <c r="AN44" t="s" s="2">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -6855,19 +6859,19 @@
         <v>77</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="N45" t="s" s="2">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="O45" t="s" s="2">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="P45" t="s" s="2">
         <v>77</v>
@@ -6916,7 +6920,7 @@
         <v>77</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>78</v>
@@ -6925,10 +6929,10 @@
         <v>79</v>
       </c>
       <c r="AI45" t="s" s="2">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="AJ45" t="s" s="2">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="AK45" t="s" s="2">
         <v>77</v>
@@ -6945,10 +6949,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -7057,10 +7061,10 @@
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7171,14 +7175,14 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="E48" s="2"/>
       <c r="F48" t="s" s="2">
@@ -7200,10 +7204,10 @@
         <v>110</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="N48" t="s" s="2">
         <v>113</v>
@@ -7258,7 +7262,7 @@
         <v>77</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>78</v>
@@ -7287,10 +7291,10 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -7313,13 +7317,13 @@
         <v>90</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
@@ -7349,10 +7353,10 @@
         <v>156</v>
       </c>
       <c r="Y49" t="s" s="2">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="Z49" t="s" s="2">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="AA49" t="s" s="2">
         <v>77</v>
@@ -7370,7 +7374,7 @@
         <v>77</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>78</v>
@@ -7379,7 +7383,7 @@
         <v>89</v>
       </c>
       <c r="AI49" t="s" s="2">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="AJ49" t="s" s="2">
         <v>101</v>
@@ -7399,10 +7403,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -7511,10 +7515,10 @@
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -7540,10 +7544,10 @@
         <v>110</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="N51" s="2"/>
       <c r="O51" s="2"/>
@@ -7623,13 +7627,13 @@
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
+        <v>398</v>
+      </c>
+      <c r="B52" t="s" s="2">
         <v>397</v>
       </c>
-      <c r="B52" t="s" s="2">
-        <v>396</v>
-      </c>
       <c r="C52" t="s" s="2">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D52" t="s" s="2">
         <v>77</v>
@@ -7651,13 +7655,13 @@
         <v>77</v>
       </c>
       <c r="K52" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="N52" s="2"/>
       <c r="O52" s="2"/>
@@ -7729,7 +7733,7 @@
         <v>77</v>
       </c>
       <c r="AM52" t="s" s="2">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="AN52" t="s" s="2">
         <v>77</v>
@@ -7737,10 +7741,10 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -7766,16 +7770,16 @@
         <v>144</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="N53" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="O53" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="P53" t="s" s="2">
         <v>77</v>
@@ -7824,7 +7828,7 @@
         <v>77</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>78</v>
@@ -7842,10 +7846,10 @@
         <v>77</v>
       </c>
       <c r="AL53" t="s" s="2">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="AM53" t="s" s="2">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="AN53" t="s" s="2">
         <v>77</v>
@@ -7853,10 +7857,10 @@
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -7882,16 +7886,16 @@
         <v>103</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="N54" t="s" s="2">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="O54" t="s" s="2">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="P54" t="s" s="2">
         <v>77</v>
@@ -7940,7 +7944,7 @@
         <v>77</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>78</v>
@@ -7958,10 +7962,10 @@
         <v>77</v>
       </c>
       <c r="AL54" t="s" s="2">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="AM54" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="AN54" t="s" s="2">
         <v>77</v>
@@ -7969,10 +7973,10 @@
     </row>
     <row r="55">
       <c r="A55" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -7995,16 +7999,16 @@
         <v>90</v>
       </c>
       <c r="K55" t="s" s="2">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="N55" t="s" s="2">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="O55" s="2"/>
       <c r="P55" t="s" s="2">
@@ -8033,7 +8037,7 @@
         <v>156</v>
       </c>
       <c r="Y55" t="s" s="2">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="Z55" t="s" s="2">
         <v>77</v>
@@ -8042,7 +8046,7 @@
         <v>77</v>
       </c>
       <c r="AB55" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="AC55" s="2"/>
       <c r="AD55" t="s" s="2">
@@ -8052,7 +8056,7 @@
         <v>116</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>78</v>
@@ -8061,7 +8065,7 @@
         <v>89</v>
       </c>
       <c r="AI55" t="s" s="2">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="AJ55" t="s" s="2">
         <v>101</v>
@@ -8081,13 +8085,13 @@
     </row>
     <row r="56">
       <c r="A56" t="s" s="2">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C56" t="s" s="2">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="D56" t="s" s="2">
         <v>77</v>
@@ -8112,13 +8116,13 @@
         <v>103</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="M56" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="N56" t="s" s="2">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="O56" s="2"/>
       <c r="P56" t="s" s="2">
@@ -8147,7 +8151,7 @@
         <v>156</v>
       </c>
       <c r="Y56" t="s" s="2">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="Z56" t="s" s="2">
         <v>77</v>
@@ -8168,7 +8172,7 @@
         <v>77</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>78</v>
@@ -8177,13 +8181,13 @@
         <v>89</v>
       </c>
       <c r="AI56" t="s" s="2">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="AJ56" t="s" s="2">
         <v>101</v>
       </c>
       <c r="AK56" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="AL56" t="s" s="2">
         <v>77</v>
@@ -8197,10 +8201,10 @@
     </row>
     <row r="57">
       <c r="A57" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -8223,17 +8227,17 @@
         <v>90</v>
       </c>
       <c r="K57" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="M57" t="s" s="2">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="N57" s="2"/>
       <c r="O57" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="P57" t="s" s="2">
         <v>77</v>
@@ -8270,7 +8274,7 @@
         <v>77</v>
       </c>
       <c r="AB57" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="AC57" s="2"/>
       <c r="AD57" t="s" s="2">
@@ -8280,7 +8284,7 @@
         <v>116</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>78</v>
@@ -8304,18 +8308,18 @@
         <v>77</v>
       </c>
       <c r="AN57" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="2">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C58" t="s" s="2">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D58" t="s" s="2">
         <v>77</v>
@@ -8337,17 +8341,17 @@
         <v>90</v>
       </c>
       <c r="K58" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="N58" s="2"/>
       <c r="O58" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="P58" t="s" s="2">
         <v>77</v>
@@ -8396,7 +8400,7 @@
         <v>77</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>78</v>
@@ -8411,7 +8415,7 @@
         <v>101</v>
       </c>
       <c r="AK58" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="AL58" t="s" s="2">
         <v>77</v>
@@ -8420,15 +8424,15 @@
         <v>77</v>
       </c>
       <c r="AN58" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -8451,16 +8455,16 @@
         <v>90</v>
       </c>
       <c r="K59" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="L59" t="s" s="2">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="N59" t="s" s="2">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="O59" s="2"/>
       <c r="P59" t="s" s="2">
@@ -8510,7 +8514,7 @@
         <v>77</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>78</v>
@@ -8534,15 +8538,15 @@
         <v>77</v>
       </c>
       <c r="AN59" t="s" s="2">
-        <v>427</v>
+        <v>428</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s" s="2">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -8568,13 +8572,13 @@
         <v>103</v>
       </c>
       <c r="L60" t="s" s="2">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="M60" t="s" s="2">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="N60" t="s" s="2">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="O60" s="2"/>
       <c r="P60" t="s" s="2">
@@ -8624,7 +8628,7 @@
         <v>77</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>78</v>
@@ -8653,10 +8657,10 @@
     </row>
     <row r="61">
       <c r="A61" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -8679,16 +8683,16 @@
         <v>90</v>
       </c>
       <c r="K61" t="s" s="2">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="L61" t="s" s="2">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="M61" t="s" s="2">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="N61" t="s" s="2">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="O61" s="2"/>
       <c r="P61" t="s" s="2">
@@ -8738,7 +8742,7 @@
         <v>77</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>78</v>
@@ -8762,15 +8766,15 @@
         <v>77</v>
       </c>
       <c r="AN61" t="s" s="2">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s" s="2">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -8793,17 +8797,17 @@
         <v>77</v>
       </c>
       <c r="K62" t="s" s="2">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="L62" t="s" s="2">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="M62" t="s" s="2">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="N62" s="2"/>
       <c r="O62" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="P62" t="s" s="2">
         <v>77</v>
@@ -8852,7 +8856,7 @@
         <v>77</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>78</v>
@@ -8873,18 +8877,18 @@
         <v>77</v>
       </c>
       <c r="AM62" t="s" s="2">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="AN62" t="s" s="2">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -8907,19 +8911,19 @@
         <v>77</v>
       </c>
       <c r="K63" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="L63" t="s" s="2">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="M63" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="N63" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="O63" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="P63" t="s" s="2">
         <v>77</v>
@@ -8968,7 +8972,7 @@
         <v>77</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>78</v>
@@ -8986,10 +8990,10 @@
         <v>77</v>
       </c>
       <c r="AL63" t="s" s="2">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="AM63" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="AN63" t="s" s="2">
         <v>77</v>
@@ -8997,10 +9001,10 @@
     </row>
     <row r="64">
       <c r="A64" t="s" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -9023,19 +9027,19 @@
         <v>77</v>
       </c>
       <c r="K64" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="L64" t="s" s="2">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="M64" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="N64" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="O64" t="s" s="2">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="P64" t="s" s="2">
         <v>77</v>
@@ -9063,10 +9067,10 @@
         <v>156</v>
       </c>
       <c r="Y64" t="s" s="2">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="Z64" t="s" s="2">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="AA64" t="s" s="2">
         <v>77</v>
@@ -9084,7 +9088,7 @@
         <v>77</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>78</v>
@@ -9113,10 +9117,10 @@
     </row>
     <row r="65">
       <c r="A65" t="s" s="2">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -9139,19 +9143,19 @@
         <v>77</v>
       </c>
       <c r="K65" t="s" s="2">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="L65" t="s" s="2">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="M65" t="s" s="2">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="N65" t="s" s="2">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="O65" t="s" s="2">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="P65" t="s" s="2">
         <v>77</v>
@@ -9200,7 +9204,7 @@
         <v>77</v>
       </c>
       <c r="AF65" t="s" s="2">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="AG65" t="s" s="2">
         <v>78</v>

</xml_diff>